<commit_message>
Extend fixture 06: two-sheet workbook with diagonal multi-table layout
Sheet '2026' (active): original Hardware/Software table unchanged.
Sheet '2025': 3 side-by-side tables shifted diagonally, each adding an
'Others' category and doubling prices (×1/×2/×4). Pattern updated from
table:1 to table:* so the engine extracts all three instances. Generator
and integration tests (TestMergedCells + TestMergedCells2025) updated to
match. 319 tests pass.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/06_merged_cells/data.xlsx
+++ b/tests/fixtures/06_merged_cells/data.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2026" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2025" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -528,4 +529,463 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SALES CATALOGUE 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Laptop 15"</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Wireless Mouse</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>29.99</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>89.98999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Office Suite</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Design Suite</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dev Tools</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>other-1</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>other-2</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>other-3</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>other-4</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3369.98</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Laptop 15"</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Wireless Mouse</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>59.98</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>179.98</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Office Suite</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Design Suite</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Dev Tools</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>other-1</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>other-2</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>other-3</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>other-4</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>6739.96</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Laptop 15"</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>4800</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Wireless Mouse</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>119.96</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Keyboard</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>359.96</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Office Suite</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Design Suite</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2400</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Dev Tools</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Others</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>other-1</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>other-2</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>other-3</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>other-4</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>13479.92</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A9:A12"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D39:D42"/>
+    <mergeCell ref="C25:C28"/>
+    <mergeCell ref="A3:A5"/>
+    <mergeCell ref="C19:C21"/>
+    <mergeCell ref="C22:C24"/>
+    <mergeCell ref="D33:D35"/>
+    <mergeCell ref="A6:A8"/>
+    <mergeCell ref="D36:D38"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>